<commit_message>
fix: move alarm parser files to correct spar/ subdirectory
Previous merge placed files at repo-root level (remote_work/src/ etc.)
instead of spar/src/ due to worktree path mismatch. Move to correct paths.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/spar/data/samples/alarm_excel_ref_sample.xlsx
+++ b/spar/data/samples/alarm_excel_ref_sample.xlsx
@@ -7,7 +7,9 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="alarms" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Guide" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RAN Alarms" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Non-RAN Alarms" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -17,13 +19,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -46,8 +51,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,40 +419,90 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Alarm ID</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
+          <t>Samsung RAN Alarm Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Sheet structure:</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sheet 1 — RAN Alarms     : code format A + 7 digits + R</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Sheet 2 — Non-RAN Alarms : code format [AH] + 3 digits + D</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr"/>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Column order: Alarm Code | Alarm Name | Severity | Group</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Alarm Code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>Alarm Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>Category</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>Module</t>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Group</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ALM-1001</t>
+          <t>A0010001R</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -462,18 +518,13 @@
       <c r="D2" t="inlineStr">
         <is>
           <t>Radio</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>gNB-DU</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>ALM-1002</t>
+          <t>A0010002R</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -489,18 +540,13 @@
       <c r="D3" t="inlineStr">
         <is>
           <t>Transport</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>gNB-CU</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>ALM-1003</t>
+          <t>A0010003R</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -516,18 +562,13 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>Radio</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>gNB-DU</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>ALM-1004</t>
+          <t>A0010004R</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -543,18 +584,13 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>HW</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>RU</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>ALM-1005</t>
+          <t>A0010005R</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -570,18 +606,13 @@
       <c r="D6" t="inlineStr">
         <is>
           <t>HW</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>BBU</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>ALM-1006</t>
+          <t>A0010006R</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -597,23 +628,18 @@
       <c r="D7" t="inlineStr">
         <is>
           <t>Transport</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>gNB-DU</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ALM-1007</t>
+          <t>A0010007R</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>License Expiring</t>
+          <t>PRACH Anomaly</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -623,147 +649,241 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>SW</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>OAM</t>
+          <t>Radio</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ALM-1008</t>
+          <t>A0010008R</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>Power Redundancy Lost</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Alarm Code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Alarm Name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Group</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>A001D</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>License Expiring</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>A002D</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>High CPU Usage</t>
         </is>
       </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Minor</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>A003D</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Backup Failed</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>A004D</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Config Mismatch</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>SW</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>H001D</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>NTP Sync Loss</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sync</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>H002D</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Disk Full</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>Major</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>HW</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>H003D</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Auth Failure</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Security</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>H004D</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Certificate Expiry</t>
+        </is>
+      </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Minor</t>
+          <t>Warning</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>SW</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>gNB-CU</t>
-        </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>ALM-1009</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>PRACH Anomaly</t>
-        </is>
-      </c>
-      <c r="C10" t="inlineStr">
-        <is>
-          <t>Minor</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Radio</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>gNB-DU</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>ALM-1010</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Backup Failed</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>SW</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>OAM</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>ALM-1011</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>Config Mismatch</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>Warning</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>SW</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>gNB-CU</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>ALM-1012</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>Power Redundancy Lost</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>Major</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>HW</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>BBU</t>
+          <t>Security</t>
         </is>
       </c>
     </row>

</xml_diff>